<commit_message>
Added updated entity file
</commit_message>
<xml_diff>
--- a/Návrh entit.xlsx
+++ b/Návrh entit.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30602"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="43" documentId="11_9248850502FE1862EC150658873E8C1851038383" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EDC20F62-F899-45A4-B0BF-F0DFA37BAD8C}"/>
+  <xr:revisionPtr revIDLastSave="116" documentId="11_9248850502FE1862EC150658873E8C1851038383" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BBB1C394-A27E-4BE0-85F9-3D79410D57D4}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,18 +34,45 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="33">
+  <si>
+    <t>Type</t>
+  </si>
   <si>
     <t>Location</t>
   </si>
   <si>
+    <t>TypeID</t>
+  </si>
+  <si>
+    <t>1:N</t>
+  </si>
+  <si>
+    <t>LocationID</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>User</t>
+  </si>
+  <si>
+    <t>TypeName</t>
+  </si>
+  <si>
     <t>Image</t>
   </si>
   <si>
-    <t>Comment</t>
-  </si>
-  <si>
-    <t>Type (location/interactive</t>
+    <t>CommentID</t>
+  </si>
+  <si>
+    <t>N:1</t>
+  </si>
+  <si>
+    <t>UserID</t>
+  </si>
+  <si>
+    <t>Type (location/interactive)</t>
   </si>
   <si>
     <t>Username</t>
@@ -54,35 +81,65 @@
     <t>Kind (shop, casino, monument, etc)</t>
   </si>
   <si>
-    <t>1:N</t>
-  </si>
-  <si>
     <t>Content</t>
   </si>
   <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Kind</t>
+  </si>
+  <si>
     <t>Date and time</t>
   </si>
   <si>
+    <t>First name</t>
+  </si>
+  <si>
+    <t>KindID</t>
+  </si>
+  <si>
     <t>Name</t>
   </si>
   <si>
     <t>Location (nav property)</t>
   </si>
   <si>
+    <t>Last name</t>
+  </si>
+  <si>
+    <t>KindName</t>
+  </si>
+  <si>
     <t>Location/Address</t>
   </si>
   <si>
+    <t>Address</t>
+  </si>
+  <si>
     <t>Visited</t>
   </si>
   <si>
+    <t>City</t>
+  </si>
+  <si>
     <t>Coords on map</t>
+  </si>
+  <si>
+    <t>Zip code</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>Balance</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -97,6 +154,14 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -106,7 +171,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -153,11 +218,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -171,7 +251,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -195,16 +278,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>2190750</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>2038350</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>2019300</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -221,8 +304,182 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm flipV="1">
-          <a:off x="4238625" y="981075"/>
-          <a:ext cx="2057400" cy="0"/>
+          <a:off x="6467475" y="561975"/>
+          <a:ext cx="1962150" cy="685800"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>28575</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2095500</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="3" name="Přímá spojnice 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{417D251F-BE92-5B8F-E6E9-BB2BBE8B9BF4}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{46270633-9401-60E0-0EA1-F1D9C77EF43C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:cxnSpLocks/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2076450" y="323850"/>
+          <a:ext cx="2066925" cy="495300"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>2143125</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="4" name="Přímá spojnice 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{20040C05-A3E6-08D6-2D6F-2D54F459ED4B}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{417D251F-BE92-5B8F-E6E9-BB2BBE8B9BF4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:cxnSpLocks/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="2114550" y="1095375"/>
+          <a:ext cx="2076450" cy="171450"/>
+        </a:xfrm>
+        <a:prstGeom prst="line">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="dk1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="dk1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>38100</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>2009775</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="5" name="Přímá spojnice 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{52A8C89C-A036-80BD-2A81-8C3587FEF85D}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{20040C05-A3E6-08D6-2D6F-2D54F459ED4B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr>
+          <a:cxnSpLocks/>
+        </xdr:cNvCxnSpPr>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="10544175" y="838200"/>
+          <a:ext cx="1971675" cy="57150"/>
         </a:xfrm>
         <a:prstGeom prst="line">
           <a:avLst/>
@@ -548,75 +805,148 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:D10"/>
+  <dimension ref="A2:G13"/>
   <sheetFormatPr defaultColWidth="30.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30.7109375" style="1"/>
-    <col min="2" max="2" width="33.140625" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="30.7109375" style="1"/>
+    <col min="2" max="2" width="32.85546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="32.5703125" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="30.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4">
-      <c r="B2" s="4" t="s">
+    <row r="2" spans="1:7">
+      <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="2:4">
-      <c r="B3" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="5" t="s">
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="2:4">
-      <c r="B4" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="2:4">
-      <c r="B5" s="2" t="s">
+      <c r="E3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="G3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="2" t="s">
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="2:4">
-      <c r="B6" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D6" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" spans="2:4">
-      <c r="B7" s="2" t="s">
+      <c r="D4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="F4" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="8" spans="2:4">
-      <c r="B8" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="2:4">
-      <c r="B9" s="2" t="s">
+    <row r="5" spans="1:7">
+      <c r="C5" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="10" spans="2:4">
-      <c r="B10" s="3" t="s">
+      <c r="E5" s="2" t="s">
         <v>13</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="B6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="C10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="C11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="G12" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="G13" s="3" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>